<commit_message>
WAM scenario for iMACC
Add WAM scenarios and corrections into growth constraints to enable the scenarios
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_B_SYS_MaxGrowthRates.xlsx
+++ b/SuppXLS/Scen_B_SYS_MaxGrowthRates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rbsul\Documents\GitHub\times-ireland-model\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CC99A54-7941-4404-8823-90981A0238ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79F55FFC-A9DF-4B25-ABDF-484619F8EE69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="8" xr2:uid="{39DC52AD-7AD8-48BE-9D85-AA1C40791A2D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{39DC52AD-7AD8-48BE-9D85-AA1C40791A2D}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="6" r:id="rId1"/>
@@ -4032,6 +4032,9 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -4040,9 +4043,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1680">
@@ -6464,17 +6464,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F13930EE-8DBF-4E65-B94E-3B7AE49D01AA}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:Z99"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="4" width="21.7265625" customWidth="1"/>
-    <col min="5" max="6" width="14.26953125" customWidth="1"/>
-    <col min="7" max="7" width="12.26953125" customWidth="1"/>
-    <col min="8" max="10" width="8.26953125" customWidth="1"/>
-    <col min="11" max="11" width="9.7265625" customWidth="1"/>
-    <col min="12" max="12" width="8.26953125" customWidth="1"/>
+    <col min="1" max="4" width="21.7109375" customWidth="1"/>
+    <col min="5" max="6" width="14.28515625" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" customWidth="1"/>
+    <col min="8" max="10" width="8.28515625" customWidth="1"/>
+    <col min="11" max="11" width="9.7109375" customWidth="1"/>
+    <col min="12" max="12" width="8.28515625" customWidth="1"/>
     <col min="13" max="13" width="10" customWidth="1"/>
-    <col min="14" max="14" width="11.453125" customWidth="1"/>
-    <col min="15" max="15" width="13.453125" customWidth="1"/>
+    <col min="14" max="14" width="11.42578125" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26">
@@ -6898,12 +6898,12 @@
       <c r="Z15" s="31"/>
     </row>
     <row r="16" spans="1:26" ht="102.75" customHeight="1">
-      <c r="A16" s="72" t="s">
+      <c r="A16" s="73" t="s">
         <v>161</v>
       </c>
-      <c r="B16" s="72"/>
-      <c r="C16" s="72"/>
-      <c r="D16" s="72"/>
+      <c r="B16" s="73"/>
+      <c r="C16" s="73"/>
+      <c r="D16" s="73"/>
       <c r="E16" s="32"/>
       <c r="F16" s="32"/>
       <c r="G16" s="33"/>
@@ -6987,11 +6987,11 @@
       <c r="A19" s="37" t="s">
         <v>162</v>
       </c>
-      <c r="B19" s="71" t="s">
+      <c r="B19" s="72" t="s">
         <v>173</v>
       </c>
-      <c r="C19" s="71"/>
-      <c r="D19" s="71"/>
+      <c r="C19" s="72"/>
+      <c r="D19" s="72"/>
       <c r="E19" s="38"/>
       <c r="F19" s="38"/>
       <c r="G19" s="39"/>
@@ -7019,11 +7019,11 @@
       <c r="A20" s="37" t="s">
         <v>163</v>
       </c>
-      <c r="B20" s="71" t="s">
+      <c r="B20" s="72" t="s">
         <v>176</v>
       </c>
-      <c r="C20" s="71"/>
-      <c r="D20" s="71"/>
+      <c r="C20" s="72"/>
+      <c r="D20" s="72"/>
       <c r="E20" s="38"/>
       <c r="F20" s="38"/>
       <c r="G20" s="39"/>
@@ -7111,11 +7111,11 @@
       <c r="A23" s="37" t="s">
         <v>165</v>
       </c>
-      <c r="B23" s="71" t="s">
+      <c r="B23" s="72" t="s">
         <v>178</v>
       </c>
-      <c r="C23" s="71"/>
-      <c r="D23" s="71"/>
+      <c r="C23" s="72"/>
+      <c r="D23" s="72"/>
       <c r="E23" s="31"/>
       <c r="F23" s="31"/>
       <c r="G23" s="31"/>
@@ -7141,11 +7141,11 @@
     </row>
     <row r="24" spans="1:26" ht="17.25" customHeight="1">
       <c r="A24" s="37"/>
-      <c r="B24" s="71" t="s">
+      <c r="B24" s="72" t="s">
         <v>174</v>
       </c>
-      <c r="C24" s="71"/>
-      <c r="D24" s="71"/>
+      <c r="C24" s="72"/>
+      <c r="D24" s="72"/>
       <c r="E24" s="31"/>
       <c r="F24" s="31"/>
       <c r="G24" s="31"/>
@@ -7203,11 +7203,11 @@
       <c r="A26" s="37" t="s">
         <v>166</v>
       </c>
-      <c r="B26" s="71" t="s">
+      <c r="B26" s="72" t="s">
         <v>242</v>
       </c>
-      <c r="C26" s="71"/>
-      <c r="D26" s="71"/>
+      <c r="C26" s="72"/>
+      <c r="D26" s="72"/>
       <c r="E26" s="31"/>
       <c r="F26" s="31"/>
       <c r="G26" s="31"/>
@@ -7233,11 +7233,11 @@
     </row>
     <row r="27" spans="1:26" ht="17.25" customHeight="1">
       <c r="A27" s="37"/>
-      <c r="B27" s="71" t="s">
+      <c r="B27" s="72" t="s">
         <v>174</v>
       </c>
-      <c r="C27" s="71"/>
-      <c r="D27" s="71"/>
+      <c r="C27" s="72"/>
+      <c r="D27" s="72"/>
       <c r="E27" s="31"/>
       <c r="F27" s="31"/>
       <c r="G27" s="31"/>
@@ -7325,11 +7325,11 @@
       <c r="A30" s="37" t="s">
         <v>168</v>
       </c>
-      <c r="B30" s="73" t="s">
+      <c r="B30" s="74" t="s">
         <v>169</v>
       </c>
-      <c r="C30" s="71"/>
-      <c r="D30" s="71"/>
+      <c r="C30" s="72"/>
+      <c r="D30" s="72"/>
       <c r="E30" s="42"/>
       <c r="F30" s="42"/>
       <c r="G30" s="31"/>
@@ -7357,11 +7357,11 @@
       <c r="A31" s="37" t="s">
         <v>170</v>
       </c>
-      <c r="B31" s="71" t="s">
+      <c r="B31" s="72" t="s">
         <v>171</v>
       </c>
-      <c r="C31" s="71"/>
-      <c r="D31" s="71"/>
+      <c r="C31" s="72"/>
+      <c r="D31" s="72"/>
       <c r="E31" s="42"/>
       <c r="F31" s="42"/>
       <c r="G31" s="31"/>
@@ -9317,35 +9317,35 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E206C345-0D8E-4CDB-A3D4-9EEBCC27251E}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A3:AD37"/>
-  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.26953125" customWidth="1"/>
-    <col min="2" max="2" width="11.7265625" customWidth="1"/>
-    <col min="3" max="3" width="3.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="5.7265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="5.7265625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.26953125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.7265625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.54296875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.26953125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="5.7265625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.26953125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="5.7265625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="5.54296875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.7265625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.7265625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="4.7265625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="7.54296875" customWidth="1"/>
-    <col min="25" max="25" width="6.7265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.28515625" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="7.5703125" customWidth="1"/>
+    <col min="25" max="25" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="27" max="28" width="6" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="5.7265625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="6.7265625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="6.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:30">
@@ -9816,7 +9816,7 @@
         <v>IE-MN</v>
       </c>
     </row>
-    <row r="10" spans="1:30" ht="15" thickBot="1">
+    <row r="10" spans="1:30" ht="15.75" thickBot="1">
       <c r="A10" s="22" t="s">
         <v>56</v>
       </c>
@@ -10075,15 +10075,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89417C8F-9D07-4311-9372-0B0C534E50C4}">
   <dimension ref="A2:N32"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="27.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.453125" customWidth="1"/>
-    <col min="11" max="11" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="39.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" customWidth="1"/>
+    <col min="11" max="11" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="39.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:14">
@@ -10387,7 +10387,7 @@
       </c>
       <c r="H20" s="46"/>
     </row>
-    <row r="21" spans="1:12" ht="15" thickBot="1">
+    <row r="21" spans="1:12" ht="15.75" thickBot="1">
       <c r="B21" s="47" t="s">
         <v>216</v>
       </c>
@@ -10641,16 +10641,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43B92B0C-7472-4C75-A119-CE0EE6C8A8E0}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A2:Z66"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.26953125" customWidth="1"/>
-    <col min="10" max="10" width="14.453125" customWidth="1"/>
-    <col min="11" max="11" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="39.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" customWidth="1"/>
+    <col min="10" max="10" width="14.42578125" customWidth="1"/>
+    <col min="11" max="11" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="39.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:26">
@@ -11338,8 +11338,8 @@
         <v>1</v>
       </c>
       <c r="H29" s="61">
-        <f>6.4-5.755</f>
-        <v>0.64500000000000046</v>
+        <f>H28+0.2</f>
+        <v>0.86499999999999999</v>
       </c>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
@@ -11361,8 +11361,8 @@
         <v>1</v>
       </c>
       <c r="H30" s="61">
-        <f>+H29</f>
-        <v>0.64500000000000046</v>
+        <f>H29+0.2</f>
+        <v>1.0649999999999999</v>
       </c>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
@@ -11384,8 +11384,8 @@
         <v>1</v>
       </c>
       <c r="H31" s="63">
-        <f>+H30</f>
-        <v>0.64500000000000046</v>
+        <f>H30+0.2</f>
+        <v>1.2649999999999999</v>
       </c>
       <c r="I31" s="18"/>
       <c r="J31" s="18"/>
@@ -11557,9 +11557,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10721BC9-19B1-4D97-BFD3-7736E255AD14}">
   <dimension ref="B2:R31"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="27.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:14">
@@ -12261,20 +12261,20 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9933FEB4-63EA-406B-A848-C3344FC12632}">
   <dimension ref="A2:N37"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="32.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.7265625" customWidth="1"/>
-    <col min="7" max="7" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.26953125" customWidth="1"/>
-    <col min="9" max="9" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.26953125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="38.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" customWidth="1"/>
+    <col min="7" max="7" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.28515625" customWidth="1"/>
+    <col min="9" max="9" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="38.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:14">
@@ -13045,7 +13045,7 @@
       </c>
       <c r="H35" s="46"/>
     </row>
-    <row r="36" spans="2:8" ht="15" thickBot="1">
+    <row r="36" spans="2:8" ht="15.75" thickBot="1">
       <c r="B36" s="47" t="s">
         <v>216</v>
       </c>
@@ -13098,19 +13098,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5F46D0-BFBE-459D-AD94-C3EBC85EC70F}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A2:N24"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="32.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.7265625" customWidth="1"/>
-    <col min="7" max="7" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.26953125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.7109375" customWidth="1"/>
+    <col min="7" max="7" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="40" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -13503,7 +13503,7 @@
       <c r="B22" s="45"/>
       <c r="H22" s="46"/>
     </row>
-    <row r="23" spans="1:8" ht="15" thickBot="1">
+    <row r="23" spans="1:8" ht="15.75" thickBot="1">
       <c r="B23" s="47" t="s">
         <v>216</v>
       </c>
@@ -13555,19 +13555,19 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6663777E-BCE4-472D-B253-88326C1C4E47}">
   <dimension ref="A2:N10"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="32.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.26953125" customWidth="1"/>
-    <col min="9" max="9" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.7265625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="38.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.28515625" customWidth="1"/>
+    <col min="9" max="9" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="38.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:14">
@@ -13762,22 +13762,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A41B7AF2-8905-43A5-8387-D99F068F4BCD}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A2:P68"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="29.7265625" customWidth="1"/>
-    <col min="3" max="3" width="14.26953125" customWidth="1"/>
+    <col min="2" max="2" width="29.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="11.26953125" customWidth="1"/>
-    <col min="6" max="6" width="10.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.26953125" customWidth="1"/>
-    <col min="8" max="8" width="10.26953125" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.54296875" customWidth="1"/>
-    <col min="14" max="14" width="13.54296875" customWidth="1"/>
-    <col min="15" max="15" width="10.7265625" customWidth="1"/>
-    <col min="16" max="16" width="11.26953125" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" customWidth="1"/>
+    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" customWidth="1"/>
+    <col min="8" max="8" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.5703125" customWidth="1"/>
+    <col min="14" max="14" width="13.5703125" customWidth="1"/>
+    <col min="15" max="15" width="10.7109375" customWidth="1"/>
+    <col min="16" max="16" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:15">
@@ -13940,14 +13940,13 @@
         <v>15</v>
       </c>
       <c r="J7" s="26">
-        <f t="shared" ref="J7:J25" si="1">1+$K30</f>
-        <v>1.8</v>
+        <v>4</v>
       </c>
       <c r="K7" s="2">
         <v>1</v>
       </c>
       <c r="L7" s="16">
-        <f t="shared" ref="L7:L11" si="2">-$B$59*L30/1000</f>
+        <f>-$B$59*L30/1000</f>
         <v>-24.2242</v>
       </c>
       <c r="M7" s="2">
@@ -13981,14 +13980,14 @@
         <v>15</v>
       </c>
       <c r="J8" s="26">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="J8:J25" si="1">1+$K31</f>
         <v>1.5</v>
       </c>
       <c r="K8" s="2">
         <v>1</v>
       </c>
       <c r="L8" s="16">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="L8:L11" si="2">-$B$59*L31/1000</f>
         <v>-24.2242</v>
       </c>
       <c r="M8" s="2">
@@ -14739,7 +14738,7 @@
         <v>130</v>
       </c>
       <c r="K30" s="11">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="L30" s="11">
         <v>0.2</v>
@@ -14771,7 +14770,7 @@
       </c>
     </row>
     <row r="32" spans="1:15">
-      <c r="A32" s="74" t="s">
+      <c r="A32" s="71" t="s">
         <v>27</v>
       </c>
       <c r="B32" t="s">
@@ -14801,7 +14800,7 @@
       </c>
     </row>
     <row r="33" spans="1:12">
-      <c r="A33" s="74"/>
+      <c r="A33" s="71"/>
       <c r="B33" t="s">
         <v>25</v>
       </c>
@@ -14829,7 +14828,7 @@
       </c>
     </row>
     <row r="34" spans="1:12">
-      <c r="A34" s="74"/>
+      <c r="A34" s="71"/>
       <c r="B34" t="s">
         <v>24</v>
       </c>
@@ -14857,7 +14856,7 @@
       </c>
     </row>
     <row r="35" spans="1:12">
-      <c r="A35" s="74"/>
+      <c r="A35" s="71"/>
       <c r="B35" t="s">
         <v>23</v>
       </c>
@@ -14885,7 +14884,7 @@
       </c>
     </row>
     <row r="36" spans="1:12">
-      <c r="A36" s="74"/>
+      <c r="A36" s="71"/>
       <c r="B36" t="s">
         <v>22</v>
       </c>
@@ -14913,7 +14912,7 @@
       </c>
     </row>
     <row r="37" spans="1:12">
-      <c r="A37" s="74"/>
+      <c r="A37" s="71"/>
       <c r="B37" t="s">
         <v>21</v>
       </c>

</xml_diff>

<commit_message>
Final MACC run changes
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_B_SYS_MaxGrowthRates.xlsx
+++ b/SuppXLS/Scen_B_SYS_MaxGrowthRates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rbsul\Documents\GitHub\times-ireland-model\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79F55FFC-A9DF-4B25-ABDF-484619F8EE69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94767615-02FA-46B7-B69C-D3204EB09039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{39DC52AD-7AD8-48BE-9D85-AA1C40791A2D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="5" xr2:uid="{39DC52AD-7AD8-48BE-9D85-AA1C40791A2D}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="6" r:id="rId1"/>
@@ -4032,9 +4032,6 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -4043,6 +4040,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1680">
@@ -6464,17 +6464,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F13930EE-8DBF-4E65-B94E-3B7AE49D01AA}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:Z99"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="4" width="21.7109375" customWidth="1"/>
-    <col min="5" max="6" width="14.28515625" customWidth="1"/>
-    <col min="7" max="7" width="12.28515625" customWidth="1"/>
-    <col min="8" max="10" width="8.28515625" customWidth="1"/>
-    <col min="11" max="11" width="9.7109375" customWidth="1"/>
-    <col min="12" max="12" width="8.28515625" customWidth="1"/>
+    <col min="1" max="4" width="21.7265625" customWidth="1"/>
+    <col min="5" max="6" width="14.26953125" customWidth="1"/>
+    <col min="7" max="7" width="12.26953125" customWidth="1"/>
+    <col min="8" max="10" width="8.26953125" customWidth="1"/>
+    <col min="11" max="11" width="9.7265625" customWidth="1"/>
+    <col min="12" max="12" width="8.26953125" customWidth="1"/>
     <col min="13" max="13" width="10" customWidth="1"/>
-    <col min="14" max="14" width="11.42578125" customWidth="1"/>
-    <col min="15" max="15" width="13.42578125" customWidth="1"/>
+    <col min="14" max="14" width="11.453125" customWidth="1"/>
+    <col min="15" max="15" width="13.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26">
@@ -6898,12 +6898,12 @@
       <c r="Z15" s="31"/>
     </row>
     <row r="16" spans="1:26" ht="102.75" customHeight="1">
-      <c r="A16" s="73" t="s">
+      <c r="A16" s="72" t="s">
         <v>161</v>
       </c>
-      <c r="B16" s="73"/>
-      <c r="C16" s="73"/>
-      <c r="D16" s="73"/>
+      <c r="B16" s="72"/>
+      <c r="C16" s="72"/>
+      <c r="D16" s="72"/>
       <c r="E16" s="32"/>
       <c r="F16" s="32"/>
       <c r="G16" s="33"/>
@@ -6987,11 +6987,11 @@
       <c r="A19" s="37" t="s">
         <v>162</v>
       </c>
-      <c r="B19" s="72" t="s">
+      <c r="B19" s="71" t="s">
         <v>173</v>
       </c>
-      <c r="C19" s="72"/>
-      <c r="D19" s="72"/>
+      <c r="C19" s="71"/>
+      <c r="D19" s="71"/>
       <c r="E19" s="38"/>
       <c r="F19" s="38"/>
       <c r="G19" s="39"/>
@@ -7019,11 +7019,11 @@
       <c r="A20" s="37" t="s">
         <v>163</v>
       </c>
-      <c r="B20" s="72" t="s">
+      <c r="B20" s="71" t="s">
         <v>176</v>
       </c>
-      <c r="C20" s="72"/>
-      <c r="D20" s="72"/>
+      <c r="C20" s="71"/>
+      <c r="D20" s="71"/>
       <c r="E20" s="38"/>
       <c r="F20" s="38"/>
       <c r="G20" s="39"/>
@@ -7111,11 +7111,11 @@
       <c r="A23" s="37" t="s">
         <v>165</v>
       </c>
-      <c r="B23" s="72" t="s">
+      <c r="B23" s="71" t="s">
         <v>178</v>
       </c>
-      <c r="C23" s="72"/>
-      <c r="D23" s="72"/>
+      <c r="C23" s="71"/>
+      <c r="D23" s="71"/>
       <c r="E23" s="31"/>
       <c r="F23" s="31"/>
       <c r="G23" s="31"/>
@@ -7141,11 +7141,11 @@
     </row>
     <row r="24" spans="1:26" ht="17.25" customHeight="1">
       <c r="A24" s="37"/>
-      <c r="B24" s="72" t="s">
+      <c r="B24" s="71" t="s">
         <v>174</v>
       </c>
-      <c r="C24" s="72"/>
-      <c r="D24" s="72"/>
+      <c r="C24" s="71"/>
+      <c r="D24" s="71"/>
       <c r="E24" s="31"/>
       <c r="F24" s="31"/>
       <c r="G24" s="31"/>
@@ -7203,11 +7203,11 @@
       <c r="A26" s="37" t="s">
         <v>166</v>
       </c>
-      <c r="B26" s="72" t="s">
+      <c r="B26" s="71" t="s">
         <v>242</v>
       </c>
-      <c r="C26" s="72"/>
-      <c r="D26" s="72"/>
+      <c r="C26" s="71"/>
+      <c r="D26" s="71"/>
       <c r="E26" s="31"/>
       <c r="F26" s="31"/>
       <c r="G26" s="31"/>
@@ -7233,11 +7233,11 @@
     </row>
     <row r="27" spans="1:26" ht="17.25" customHeight="1">
       <c r="A27" s="37"/>
-      <c r="B27" s="72" t="s">
+      <c r="B27" s="71" t="s">
         <v>174</v>
       </c>
-      <c r="C27" s="72"/>
-      <c r="D27" s="72"/>
+      <c r="C27" s="71"/>
+      <c r="D27" s="71"/>
       <c r="E27" s="31"/>
       <c r="F27" s="31"/>
       <c r="G27" s="31"/>
@@ -7325,11 +7325,11 @@
       <c r="A30" s="37" t="s">
         <v>168</v>
       </c>
-      <c r="B30" s="74" t="s">
+      <c r="B30" s="73" t="s">
         <v>169</v>
       </c>
-      <c r="C30" s="72"/>
-      <c r="D30" s="72"/>
+      <c r="C30" s="71"/>
+      <c r="D30" s="71"/>
       <c r="E30" s="42"/>
       <c r="F30" s="42"/>
       <c r="G30" s="31"/>
@@ -7357,11 +7357,11 @@
       <c r="A31" s="37" t="s">
         <v>170</v>
       </c>
-      <c r="B31" s="72" t="s">
+      <c r="B31" s="71" t="s">
         <v>171</v>
       </c>
-      <c r="C31" s="72"/>
-      <c r="D31" s="72"/>
+      <c r="C31" s="71"/>
+      <c r="D31" s="71"/>
       <c r="E31" s="42"/>
       <c r="F31" s="42"/>
       <c r="G31" s="31"/>
@@ -9317,35 +9317,35 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E206C345-0D8E-4CDB-A3D4-9EEBCC27251E}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A3:AD37"/>
-  <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12.28515625" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" customWidth="1"/>
-    <col min="3" max="3" width="3.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="4.7109375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="7.5703125" customWidth="1"/>
-    <col min="25" max="25" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.26953125" customWidth="1"/>
+    <col min="2" max="2" width="11.7265625" customWidth="1"/>
+    <col min="3" max="3" width="3.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.7265625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="5.54296875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.7265625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="4.7265625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="7.54296875" customWidth="1"/>
+    <col min="25" max="25" width="6.7265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="6.26953125" bestFit="1" customWidth="1"/>
     <col min="27" max="28" width="6" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="6.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:30">
@@ -9816,7 +9816,7 @@
         <v>IE-MN</v>
       </c>
     </row>
-    <row r="10" spans="1:30" ht="15.75" thickBot="1">
+    <row r="10" spans="1:30" ht="15" thickBot="1">
       <c r="A10" s="22" t="s">
         <v>56</v>
       </c>
@@ -10075,15 +10075,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89417C8F-9D07-4311-9372-0B0C534E50C4}">
   <dimension ref="A2:N32"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" customWidth="1"/>
-    <col min="11" max="11" width="33.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="39.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.453125" customWidth="1"/>
+    <col min="11" max="11" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="39.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:14">
@@ -10387,7 +10387,7 @@
       </c>
       <c r="H20" s="46"/>
     </row>
-    <row r="21" spans="1:12" ht="15.75" thickBot="1">
+    <row r="21" spans="1:12" ht="15" thickBot="1">
       <c r="B21" s="47" t="s">
         <v>216</v>
       </c>
@@ -10641,16 +10641,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43B92B0C-7472-4C75-A119-CE0EE6C8A8E0}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A2:Z66"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.28515625" customWidth="1"/>
-    <col min="10" max="10" width="14.42578125" customWidth="1"/>
-    <col min="11" max="11" width="33.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="39.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.26953125" customWidth="1"/>
+    <col min="10" max="10" width="14.453125" customWidth="1"/>
+    <col min="11" max="11" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="39.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:26">
@@ -11557,9 +11557,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10721BC9-19B1-4D97-BFD3-7736E255AD14}">
   <dimension ref="B2:R31"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:14">
@@ -12261,20 +12261,20 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9933FEB4-63EA-406B-A848-C3344FC12632}">
   <dimension ref="A2:N37"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.28515625" customWidth="1"/>
-    <col min="9" max="9" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="38.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.7265625" customWidth="1"/>
+    <col min="7" max="7" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.26953125" customWidth="1"/>
+    <col min="9" max="9" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="38.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:14">
@@ -12506,7 +12506,7 @@
         <v>142</v>
       </c>
       <c r="H9" s="2">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>15</v>
@@ -12546,7 +12546,7 @@
         <v>142</v>
       </c>
       <c r="H10" s="2">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>15</v>
@@ -13045,7 +13045,7 @@
       </c>
       <c r="H35" s="46"/>
     </row>
-    <row r="36" spans="2:8" ht="15.75" thickBot="1">
+    <row r="36" spans="2:8" ht="15" thickBot="1">
       <c r="B36" s="47" t="s">
         <v>216</v>
       </c>
@@ -13098,19 +13098,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5F46D0-BFBE-459D-AD94-C3EBC85EC70F}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A2:N24"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.7109375" customWidth="1"/>
-    <col min="7" max="7" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.7265625" customWidth="1"/>
+    <col min="7" max="7" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.453125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="40" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -13503,7 +13503,7 @@
       <c r="B22" s="45"/>
       <c r="H22" s="46"/>
     </row>
-    <row r="23" spans="1:8" ht="15.75" thickBot="1">
+    <row r="23" spans="1:8" ht="15" thickBot="1">
       <c r="B23" s="47" t="s">
         <v>216</v>
       </c>
@@ -13555,19 +13555,19 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6663777E-BCE4-472D-B253-88326C1C4E47}">
   <dimension ref="A2:N10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.28515625" customWidth="1"/>
-    <col min="9" max="9" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="38.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.26953125" customWidth="1"/>
+    <col min="9" max="9" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="38.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:14">
@@ -13684,7 +13684,7 @@
       </c>
       <c r="J6" s="29">
         <f>1+C10</f>
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="K6" s="2">
         <v>1</v>
@@ -13722,7 +13722,7 @@
       </c>
       <c r="K7" s="2"/>
       <c r="L7" s="16">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="M7" s="2">
         <v>5</v>
@@ -13747,7 +13747,7 @@
         <v>229</v>
       </c>
       <c r="C10" s="11">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="D10">
         <v>20</v>
@@ -13762,22 +13762,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A41B7AF2-8905-43A5-8387-D99F068F4BCD}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A2:P68"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="29.7109375" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" customWidth="1"/>
+    <col min="2" max="2" width="29.7265625" customWidth="1"/>
+    <col min="3" max="3" width="14.26953125" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" customWidth="1"/>
-    <col min="8" max="8" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.5703125" customWidth="1"/>
-    <col min="14" max="14" width="13.5703125" customWidth="1"/>
-    <col min="15" max="15" width="10.7109375" customWidth="1"/>
-    <col min="16" max="16" width="11.28515625" customWidth="1"/>
+    <col min="5" max="5" width="11.26953125" customWidth="1"/>
+    <col min="6" max="6" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.26953125" customWidth="1"/>
+    <col min="8" max="8" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.54296875" customWidth="1"/>
+    <col min="14" max="14" width="13.54296875" customWidth="1"/>
+    <col min="15" max="15" width="10.7265625" customWidth="1"/>
+    <col min="16" max="16" width="11.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:15">
@@ -14770,7 +14770,7 @@
       </c>
     </row>
     <row r="32" spans="1:15">
-      <c r="A32" s="71" t="s">
+      <c r="A32" s="74" t="s">
         <v>27</v>
       </c>
       <c r="B32" t="s">
@@ -14800,7 +14800,7 @@
       </c>
     </row>
     <row r="33" spans="1:12">
-      <c r="A33" s="71"/>
+      <c r="A33" s="74"/>
       <c r="B33" t="s">
         <v>25</v>
       </c>
@@ -14828,7 +14828,7 @@
       </c>
     </row>
     <row r="34" spans="1:12">
-      <c r="A34" s="71"/>
+      <c r="A34" s="74"/>
       <c r="B34" t="s">
         <v>24</v>
       </c>
@@ -14856,7 +14856,7 @@
       </c>
     </row>
     <row r="35" spans="1:12">
-      <c r="A35" s="71"/>
+      <c r="A35" s="74"/>
       <c r="B35" t="s">
         <v>23</v>
       </c>
@@ -14884,7 +14884,7 @@
       </c>
     </row>
     <row r="36" spans="1:12">
-      <c r="A36" s="71"/>
+      <c r="A36" s="74"/>
       <c r="B36" t="s">
         <v>22</v>
       </c>
@@ -14912,7 +14912,7 @@
       </c>
     </row>
     <row r="37" spans="1:12">
-      <c r="A37" s="71"/>
+      <c r="A37" s="74"/>
       <c r="B37" t="s">
         <v>21</v>
       </c>

</xml_diff>